<commit_message>
cierre ciclo 2026-06 — 7_cierre transiciona junio a julio
GATE (validado en 5b) → COSECHAR (foto en archivo/2026-06/, 13 archivos) →
FREEZE (estado_ciclo=CERRADO) → LIMPIAR (mesa_1..7 y correcciones_lote
reseteados a template para julio).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/4_pagos/efectivo/inputs/mesa_7.xlsx
+++ b/4_pagos/efectivo/inputs/mesa_7.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +54,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="009A3412"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001D4ED8"/>
       <sz val="10"/>
     </font>
@@ -77,12 +83,18 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009A3412"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="009CA3AF"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -109,8 +121,13 @@
         <fgColor rgb="00F4ECF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF7ED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -118,37 +135,57 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00FFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00FFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00FFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00FFFFFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -516,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -528,6 +565,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -551,96 +589,107 @@
           <t>¿Alguna nota?</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>¿Qué tipo?</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>COBRADOR</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>FECHA_REGISTRO</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>MZ</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>MONTO</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>MONTO_EFECTIVO</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>MONTO_YAPE</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>FECHA</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>COMENTARIO</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>8C</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>38.00</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>20.00</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>18.00</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>03/06/2026</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="11" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -658,7 +707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -670,6 +719,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -693,96 +743,107 @@
           <t>¿Alguna nota?</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>¿Qué tipo?</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>COBRADOR</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>FECHA_REGISTRO</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>MZ</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>MONTO</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>MONTO_EFECTIVO</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>MONTO_YAPE</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>FECHA</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>COMENTARIO</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>8C</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>38.00</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>20.00</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>18.00</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>03/06/2026</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="11" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -800,7 +861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -812,6 +873,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -835,96 +897,107 @@
           <t>¿Alguna nota?</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>¿Qué tipo?</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>COBRADOR</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>FECHA_REGISTRO</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>MZ</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>MONTO</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>MONTO_EFECTIVO</t>
         </is>
       </c>
-      <c r="G2" s="7" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>MONTO_YAPE</t>
         </is>
       </c>
-      <c r="H2" s="7" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>FECHA</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t>COMENTARIO</t>
+        </is>
+      </c>
+      <c r="J2" s="10" t="inlineStr">
+        <is>
+          <t>CONCEPTO</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>María García</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>10/06/2026</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>8C</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>38.00</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>20.00</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>18.00</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>03/06/2026</t>
         </is>
       </c>
-      <c r="I3" s="9" t="inlineStr"/>
+      <c r="I3" s="11" t="inlineStr"/>
+      <c r="J3" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>